<commit_message>
fix negative 01 TSVAL highlight
</commit_message>
<xml_diff>
--- a/rules/CORE-000468/negative/01/data/unit-test-coreid-CG0276-negative 1.xlsx
+++ b/rules/CORE-000468/negative/01/data/unit-test-coreid-CG0276-negative 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\QF\CORE\core-contributor\rules\CORE-000468\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DE7CC4F-5EF6-44BB-B984-A333F378C998}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4FB76B1-25CE-477F-ACC7-A034BD749D62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -725,7 +725,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -738,7 +738,6 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1140,6 +1139,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="5" max="5" width="31.5546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
@@ -1292,6 +1294,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K55"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="6" max="6" width="19.44140625" customWidth="1"/>
+    <col min="7" max="7" width="28.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
@@ -2605,7 +2611,7 @@
       <c r="C46" s="8">
         <v>1</v>
       </c>
-      <c r="D46" s="10" t="s">
+      <c r="D46" s="2" t="s">
         <v>46</v>
       </c>
       <c r="E46" s="7" t="s">
@@ -2823,7 +2829,7 @@
       <c r="C53" s="8">
         <v>1</v>
       </c>
-      <c r="D53" s="10" t="s">
+      <c r="D53" s="2" t="s">
         <v>46</v>
       </c>
       <c r="E53" s="4" t="s">
@@ -2832,7 +2838,7 @@
       <c r="F53" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="G53" s="4" t="s">
+      <c r="G53" s="7" t="s">
         <v>46</v>
       </c>
       <c r="H53" s="6" t="s">

</xml_diff>

<commit_message>
CG0276 address review: formatting, re-add output variables, # verified
</commit_message>
<xml_diff>
--- a/rules/CORE-000468/negative/01/data/unit-test-coreid-CG0276-negative 1.xlsx
+++ b/rules/CORE-000468/negative/01/data/unit-test-coreid-CG0276-negative 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\QF\CORE\core-contributor\rules\CORE-000468\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76341505-EB8E-4980-8E83-BEC1B4CA51C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B18DB9D-0E41-413B-BD8D-714E65C67BF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="206">
   <si>
     <t>Product</t>
   </si>
@@ -76,552 +76,555 @@
     <t>STYPE</t>
   </si>
   <si>
+    <t>TSGRPID</t>
+  </si>
+  <si>
+    <t>TSVAL</t>
+  </si>
+  <si>
+    <t>INTERVENTIONAL</t>
+  </si>
+  <si>
+    <t>$STYPE_INTERVENTIONAL</t>
+  </si>
+  <si>
+    <t>TRT</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>STUDYID</t>
+  </si>
+  <si>
+    <t>DOMAIN</t>
+  </si>
+  <si>
+    <t>TSSEQ</t>
+  </si>
+  <si>
     <t>TSPARM</t>
   </si>
   <si>
+    <t>TSVALNF</t>
+  </si>
+  <si>
+    <t>TSVALCD</t>
+  </si>
+  <si>
+    <t>TSVCDREF</t>
+  </si>
+  <si>
+    <t>TSVCDVER</t>
+  </si>
+  <si>
+    <t>Study Identifier</t>
+  </si>
+  <si>
+    <t>Domain Abbreviation</t>
+  </si>
+  <si>
+    <t>Sequence Number</t>
+  </si>
+  <si>
+    <t>Group ID</t>
+  </si>
+  <si>
+    <t>Trial Summary Parameter Short Name</t>
+  </si>
+  <si>
+    <t>Trial Summary Parameter</t>
+  </si>
+  <si>
+    <t>Parameter Value</t>
+  </si>
+  <si>
+    <t>Parameter Null Flavor</t>
+  </si>
+  <si>
+    <t>Parameter Value Code</t>
+  </si>
+  <si>
+    <t>Name of the Reference Terminology</t>
+  </si>
+  <si>
+    <t>Version of the Reference Terminology</t>
+  </si>
+  <si>
+    <t>Char</t>
+  </si>
+  <si>
+    <t>Num</t>
+  </si>
+  <si>
+    <t>CDISCPILOT01</t>
+  </si>
+  <si>
+    <t>TS</t>
+  </si>
+  <si>
+    <t>ACTSUB</t>
+  </si>
+  <si>
+    <t>Actual Number of Subjects</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>ADAPT</t>
+  </si>
+  <si>
+    <t>Adaptive Design</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>C49487</t>
+  </si>
+  <si>
+    <t>CDISC</t>
+  </si>
+  <si>
+    <t>2020-03-27</t>
+  </si>
+  <si>
+    <t>ADDON</t>
+  </si>
+  <si>
+    <t>Added on to Existing Treatments</t>
+  </si>
+  <si>
+    <t>AGEMAX</t>
+  </si>
+  <si>
+    <t>Planned Maximum Age of Subjects</t>
+  </si>
+  <si>
+    <t>PINF</t>
+  </si>
+  <si>
+    <t>AGEMIN</t>
+  </si>
+  <si>
+    <t>Planned Minimum Age of Subjects</t>
+  </si>
+  <si>
+    <t>P50Y</t>
+  </si>
+  <si>
+    <t>ISO 8601</t>
+  </si>
+  <si>
+    <t>CUTOFF</t>
+  </si>
+  <si>
+    <t>DCUTDESC</t>
+  </si>
+  <si>
+    <t>Data Cutoff Description</t>
+  </si>
+  <si>
+    <t>DATABASE LOCK</t>
+  </si>
+  <si>
+    <t>DCUTDTC</t>
+  </si>
+  <si>
+    <t>Data Cutoff Date</t>
+  </si>
+  <si>
+    <t>2015-03-31</t>
+  </si>
+  <si>
+    <t>PLACEBO</t>
+  </si>
+  <si>
+    <t>DOSE</t>
+  </si>
+  <si>
+    <t>Dose per Administration</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>LOW-DOSE</t>
+  </si>
+  <si>
+    <t>54</t>
+  </si>
+  <si>
+    <t>HIGH-DOSE</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>81</t>
+  </si>
+  <si>
+    <t>DOSFRM</t>
+  </si>
+  <si>
+    <t>Dose Form</t>
+  </si>
+  <si>
+    <t>INJECTION</t>
+  </si>
+  <si>
+    <t>C42946</t>
+  </si>
+  <si>
+    <t>DOSFRQ</t>
+  </si>
+  <si>
+    <t>Dosing Frequency</t>
+  </si>
+  <si>
+    <t>QD</t>
+  </si>
+  <si>
+    <t>C25473</t>
+  </si>
+  <si>
+    <t>DOSU</t>
+  </si>
+  <si>
+    <t>Dose Units</t>
+  </si>
+  <si>
+    <t>mg</t>
+  </si>
+  <si>
+    <t>C28253</t>
+  </si>
+  <si>
+    <t>FCNTRY</t>
+  </si>
+  <si>
+    <t>Planned Country of Investigational Sites</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>ISO 3166-1 alpha-3</t>
+  </si>
+  <si>
+    <t>HLTSUBJI</t>
+  </si>
+  <si>
+    <t>Healthy Subject Indicator</t>
+  </si>
+  <si>
+    <t>INDIC</t>
+  </si>
+  <si>
+    <t>Trial Disease/Condition Indication</t>
+  </si>
+  <si>
+    <t>Alzheimer's Disease (Disorder)</t>
+  </si>
+  <si>
+    <t>26929004</t>
+  </si>
+  <si>
+    <t>SNOMED</t>
+  </si>
+  <si>
+    <t>2019-03-01</t>
+  </si>
+  <si>
+    <t>INTMODEL</t>
+  </si>
+  <si>
+    <t>Intervention Model</t>
+  </si>
+  <si>
+    <t>PARALLEL</t>
+  </si>
+  <si>
+    <t>C82639</t>
+  </si>
+  <si>
+    <t>INTTYPE</t>
+  </si>
+  <si>
+    <t>Intervention Type</t>
+  </si>
+  <si>
+    <t>DRUG</t>
+  </si>
+  <si>
+    <t>C1909</t>
+  </si>
+  <si>
+    <t>LENGTH</t>
+  </si>
+  <si>
+    <t>Trial Length</t>
+  </si>
+  <si>
+    <t>P28W</t>
+  </si>
+  <si>
+    <t>NARMS</t>
+  </si>
+  <si>
+    <t>Planned Number of Arms</t>
+  </si>
+  <si>
+    <t>EFFICACY</t>
+  </si>
+  <si>
+    <t>OBJPRIM</t>
+  </si>
+  <si>
+    <t>Trial Primary Objective</t>
+  </si>
+  <si>
+    <t>To document the efficacy profile of Zanomaline.</t>
+  </si>
+  <si>
+    <t>SAFETY</t>
+  </si>
+  <si>
+    <t>To document the safety profile of Zanomaline.</t>
+  </si>
+  <si>
+    <t>OUTMSPRI</t>
+  </si>
+  <si>
+    <t>Primary Outcome Measure</t>
+  </si>
+  <si>
+    <t>To assess the dose-dependent improvement in subject depression. Improved scores on the Patient Health Questionnaire(PHQ-9) and the Hamilton Depression Rating Scale(HAMD 17) will indicate improvements.</t>
+  </si>
+  <si>
+    <t>To assess the dose-dependent improvements in satisfaction with subjects' lives as a whole. Improved scores on the Satisfaction With Life Survery (SWLS) will indicate improvements.</t>
+  </si>
+  <si>
+    <t>To assess the dose-dependent improvements in subject memory and learning. Improved scores on the Auditory Verbal Learning Test (AVLT-REY) will indicate improvements.</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Type, frequency, and severity of laboratory abnormalities</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Type, frequency, and severity of adverse events (AEs)</t>
+  </si>
+  <si>
+    <t>PCLAS</t>
+  </si>
+  <si>
+    <t>Pharmacologic Class</t>
+  </si>
+  <si>
+    <t>Acetylcholine Release Inhibitor</t>
+  </si>
+  <si>
+    <t>N0000175771</t>
+  </si>
+  <si>
+    <t>MED-RT</t>
+  </si>
+  <si>
+    <t>PLANSUB</t>
+  </si>
+  <si>
+    <t>Planned Number of Subjects</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>RANDOM</t>
+  </si>
+  <si>
+    <t>Trial is Randomized</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>C49488</t>
+  </si>
+  <si>
+    <t>RANDQT</t>
+  </si>
+  <si>
+    <t>Randomization Quotient</t>
+  </si>
+  <si>
+    <t>0.67</t>
+  </si>
+  <si>
+    <t>REGID</t>
+  </si>
+  <si>
+    <t>Registry Identifier</t>
+  </si>
+  <si>
+    <t>NCT00000000</t>
+  </si>
+  <si>
+    <t>clinicaltrials.gov</t>
+  </si>
+  <si>
+    <t>ROUTE</t>
+  </si>
+  <si>
+    <t>Route of Administration</t>
+  </si>
+  <si>
+    <t>SUBCUTANEOUS</t>
+  </si>
+  <si>
+    <t>C38299</t>
+  </si>
+  <si>
+    <t>SDTIGVER</t>
+  </si>
+  <si>
+    <t>SDTM IG Version</t>
+  </si>
+  <si>
+    <t>3.3</t>
+  </si>
+  <si>
+    <t>SDTMVER</t>
+  </si>
+  <si>
+    <t>SDTM Version</t>
+  </si>
+  <si>
+    <t>1.7</t>
+  </si>
+  <si>
+    <t>SENDTC</t>
+  </si>
+  <si>
+    <t>Study End Date</t>
+  </si>
+  <si>
+    <t>2014-11-01</t>
+  </si>
+  <si>
+    <t>SEXPOP</t>
+  </si>
+  <si>
+    <t>Sex of Participants</t>
+  </si>
+  <si>
+    <t>BOTH</t>
+  </si>
+  <si>
+    <t>C49636</t>
+  </si>
+  <si>
+    <t>SPONSOR</t>
+  </si>
+  <si>
+    <t>Clinical Study Sponsor</t>
+  </si>
+  <si>
+    <t>SDTM Metadata Submission Guidelines Team</t>
+  </si>
+  <si>
+    <t>SSTDTC</t>
+  </si>
+  <si>
+    <t>Study Start Date</t>
+  </si>
+  <si>
+    <t>2012-10-06</t>
+  </si>
+  <si>
+    <t>STOPRULE</t>
+  </si>
+  <si>
+    <t>Study Stop Rules</t>
+  </si>
+  <si>
+    <t>NONE</t>
+  </si>
+  <si>
     <t>Study Type</t>
   </si>
   <si>
-    <t>TSVALNF</t>
-  </si>
-  <si>
-    <t>TSVAL</t>
-  </si>
-  <si>
-    <t>INTERVENTIONAL</t>
-  </si>
-  <si>
-    <t>TRT</t>
+    <t>C98388</t>
+  </si>
+  <si>
+    <t>TBLIND</t>
+  </si>
+  <si>
+    <t>Trial Blinding Schema</t>
+  </si>
+  <si>
+    <t>DOUBLE BLIND</t>
+  </si>
+  <si>
+    <t>C15228</t>
+  </si>
+  <si>
+    <t>TCNTRL</t>
+  </si>
+  <si>
+    <t>Control Type</t>
+  </si>
+  <si>
+    <t>C49648</t>
+  </si>
+  <si>
+    <t>TDIGRP</t>
+  </si>
+  <si>
+    <t>Diagnosis Group</t>
+  </si>
+  <si>
+    <t>TINDTP</t>
+  </si>
+  <si>
+    <t>Trial Intent Type</t>
+  </si>
+  <si>
+    <t>TREATMENT</t>
+  </si>
+  <si>
+    <t>C49656</t>
+  </si>
+  <si>
+    <t>TITLE</t>
+  </si>
+  <si>
+    <t>Trial Title</t>
+  </si>
+  <si>
+    <t>Safety and Efficacy of Zanomaline in Patients with Mild to Moderate Alzheimers Disease.</t>
+  </si>
+  <si>
+    <t>TPHASE</t>
+  </si>
+  <si>
+    <t>Trial Phase Classification</t>
+  </si>
+  <si>
+    <t>PHASE II TRIAL</t>
+  </si>
+  <si>
+    <t>C15601</t>
   </si>
   <si>
     <t>Investigational Therapy or Treatment</t>
   </si>
   <si>
-    <t>STUDYID</t>
-  </si>
-  <si>
-    <t>DOMAIN</t>
-  </si>
-  <si>
-    <t>TSSEQ</t>
-  </si>
-  <si>
-    <t>TSGRPID</t>
-  </si>
-  <si>
-    <t>TSVALCD</t>
-  </si>
-  <si>
-    <t>TSVCDREF</t>
-  </si>
-  <si>
-    <t>TSVCDVER</t>
-  </si>
-  <si>
-    <t>Study Identifier</t>
-  </si>
-  <si>
-    <t>Domain Abbreviation</t>
-  </si>
-  <si>
-    <t>Sequence Number</t>
-  </si>
-  <si>
-    <t>Group ID</t>
-  </si>
-  <si>
-    <t>Trial Summary Parameter Short Name</t>
-  </si>
-  <si>
-    <t>Trial Summary Parameter</t>
-  </si>
-  <si>
-    <t>Parameter Value</t>
-  </si>
-  <si>
-    <t>Parameter Null Flavor</t>
-  </si>
-  <si>
-    <t>Parameter Value Code</t>
-  </si>
-  <si>
-    <t>Name of the Reference Terminology</t>
-  </si>
-  <si>
-    <t>Version of the Reference Terminology</t>
-  </si>
-  <si>
-    <t>Char</t>
-  </si>
-  <si>
-    <t>Num</t>
-  </si>
-  <si>
-    <t>CDISCPILOT01</t>
-  </si>
-  <si>
-    <t>TS</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>ACTSUB</t>
-  </si>
-  <si>
-    <t>Actual Number of Subjects</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>ADAPT</t>
-  </si>
-  <si>
-    <t>Adaptive Design</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>C49487</t>
-  </si>
-  <si>
-    <t>CDISC</t>
-  </si>
-  <si>
-    <t>2020-03-27</t>
-  </si>
-  <si>
-    <t>ADDON</t>
-  </si>
-  <si>
-    <t>Added on to Existing Treatments</t>
-  </si>
-  <si>
-    <t>AGEMAX</t>
-  </si>
-  <si>
-    <t>Planned Maximum Age of Subjects</t>
-  </si>
-  <si>
-    <t>PINF</t>
-  </si>
-  <si>
-    <t>AGEMIN</t>
-  </si>
-  <si>
-    <t>Planned Minimum Age of Subjects</t>
-  </si>
-  <si>
-    <t>P50Y</t>
-  </si>
-  <si>
-    <t>ISO 8601</t>
-  </si>
-  <si>
-    <t>CUTOFF</t>
-  </si>
-  <si>
-    <t>DCUTDESC</t>
-  </si>
-  <si>
-    <t>Data Cutoff Description</t>
-  </si>
-  <si>
-    <t>DATABASE LOCK</t>
-  </si>
-  <si>
-    <t>DCUTDTC</t>
-  </si>
-  <si>
-    <t>Data Cutoff Date</t>
-  </si>
-  <si>
-    <t>2015-03-31</t>
-  </si>
-  <si>
-    <t>PLACEBO</t>
-  </si>
-  <si>
-    <t>DOSE</t>
-  </si>
-  <si>
-    <t>Dose per Administration</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>LOW-DOSE</t>
-  </si>
-  <si>
-    <t>54</t>
-  </si>
-  <si>
-    <t>HIGH-DOSE</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>81</t>
-  </si>
-  <si>
-    <t>DOSFRM</t>
-  </si>
-  <si>
-    <t>Dose Form</t>
-  </si>
-  <si>
-    <t>INJECTION</t>
-  </si>
-  <si>
-    <t>C42946</t>
-  </si>
-  <si>
-    <t>DOSFRQ</t>
-  </si>
-  <si>
-    <t>Dosing Frequency</t>
-  </si>
-  <si>
-    <t>QD</t>
-  </si>
-  <si>
-    <t>C25473</t>
-  </si>
-  <si>
-    <t>DOSU</t>
-  </si>
-  <si>
-    <t>Dose Units</t>
-  </si>
-  <si>
-    <t>mg</t>
-  </si>
-  <si>
-    <t>C28253</t>
-  </si>
-  <si>
-    <t>FCNTRY</t>
-  </si>
-  <si>
-    <t>Planned Country of Investigational Sites</t>
-  </si>
-  <si>
-    <t>USA</t>
-  </si>
-  <si>
-    <t>ISO 3166-1 alpha-3</t>
-  </si>
-  <si>
-    <t>HLTSUBJI</t>
-  </si>
-  <si>
-    <t>Healthy Subject Indicator</t>
-  </si>
-  <si>
-    <t>INDIC</t>
-  </si>
-  <si>
-    <t>Trial Disease/Condition Indication</t>
-  </si>
-  <si>
-    <t>Alzheimer's Disease (Disorder)</t>
-  </si>
-  <si>
-    <t>26929004</t>
-  </si>
-  <si>
-    <t>SNOMED</t>
-  </si>
-  <si>
-    <t>2019-03-01</t>
-  </si>
-  <si>
-    <t>INTMODEL</t>
-  </si>
-  <si>
-    <t>Intervention Model</t>
-  </si>
-  <si>
-    <t>PARALLEL</t>
-  </si>
-  <si>
-    <t>C82639</t>
-  </si>
-  <si>
-    <t>INTTYPE</t>
-  </si>
-  <si>
-    <t>Intervention Type</t>
-  </si>
-  <si>
-    <t>DRUG</t>
-  </si>
-  <si>
-    <t>C1909</t>
-  </si>
-  <si>
-    <t>LENGTH</t>
-  </si>
-  <si>
-    <t>Trial Length</t>
-  </si>
-  <si>
-    <t>P28W</t>
-  </si>
-  <si>
-    <t>NARMS</t>
-  </si>
-  <si>
-    <t>Planned Number of Arms</t>
-  </si>
-  <si>
-    <t>EFFICACY</t>
-  </si>
-  <si>
-    <t>OBJPRIM</t>
-  </si>
-  <si>
-    <t>Trial Primary Objective</t>
-  </si>
-  <si>
-    <t>To document the efficacy profile of Zanomaline.</t>
-  </si>
-  <si>
-    <t>SAFETY</t>
-  </si>
-  <si>
-    <t>To document the safety profile of Zanomaline.</t>
-  </si>
-  <si>
-    <t>OUTMSPRI</t>
-  </si>
-  <si>
-    <t>Primary Outcome Measure</t>
-  </si>
-  <si>
-    <t>To assess the dose-dependent improvement in subject depression. Improved scores on the Patient Health Questionnaire(PHQ-9) and the Hamilton Depression Rating Scale(HAMD 17) will indicate improvements.</t>
-  </si>
-  <si>
-    <t>To assess the dose-dependent improvements in satisfaction with subjects' lives as a whole. Improved scores on the Satisfaction With Life Survery (SWLS) will indicate improvements.</t>
-  </si>
-  <si>
-    <t>To assess the dose-dependent improvements in subject memory and learning. Improved scores on the Auditory Verbal Learning Test (AVLT-REY) will indicate improvements.</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Type, frequency, and severity of laboratory abnormalities</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>Type, frequency, and severity of adverse events (AEs)</t>
-  </si>
-  <si>
-    <t>PCLAS</t>
-  </si>
-  <si>
-    <t>Pharmacologic Class</t>
-  </si>
-  <si>
-    <t>Acetylcholine Release Inhibitor</t>
-  </si>
-  <si>
-    <t>N0000175771</t>
-  </si>
-  <si>
-    <t>MED-RT</t>
-  </si>
-  <si>
-    <t>PLANSUB</t>
-  </si>
-  <si>
-    <t>Planned Number of Subjects</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>RANDOM</t>
-  </si>
-  <si>
-    <t>Trial is Randomized</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>C49488</t>
-  </si>
-  <si>
-    <t>RANDQT</t>
-  </si>
-  <si>
-    <t>Randomization Quotient</t>
-  </si>
-  <si>
-    <t>0.67</t>
-  </si>
-  <si>
-    <t>REGID</t>
-  </si>
-  <si>
-    <t>Registry Identifier</t>
-  </si>
-  <si>
-    <t>NCT00000000</t>
-  </si>
-  <si>
-    <t>clinicaltrials.gov</t>
-  </si>
-  <si>
-    <t>ROUTE</t>
-  </si>
-  <si>
-    <t>Route of Administration</t>
-  </si>
-  <si>
-    <t>SUBCUTANEOUS</t>
-  </si>
-  <si>
-    <t>C38299</t>
-  </si>
-  <si>
-    <t>SDTIGVER</t>
-  </si>
-  <si>
-    <t>SDTM IG Version</t>
-  </si>
-  <si>
-    <t>3.3</t>
-  </si>
-  <si>
-    <t>SDTMVER</t>
-  </si>
-  <si>
-    <t>SDTM Version</t>
-  </si>
-  <si>
-    <t>1.7</t>
-  </si>
-  <si>
-    <t>SENDTC</t>
-  </si>
-  <si>
-    <t>Study End Date</t>
-  </si>
-  <si>
-    <t>2014-11-01</t>
-  </si>
-  <si>
-    <t>SEXPOP</t>
-  </si>
-  <si>
-    <t>Sex of Participants</t>
-  </si>
-  <si>
-    <t>BOTH</t>
-  </si>
-  <si>
-    <t>C49636</t>
-  </si>
-  <si>
-    <t>SPONSOR</t>
-  </si>
-  <si>
-    <t>Clinical Study Sponsor</t>
-  </si>
-  <si>
-    <t>SDTM Metadata Submission Guidelines Team</t>
-  </si>
-  <si>
-    <t>SSTDTC</t>
-  </si>
-  <si>
-    <t>Study Start Date</t>
-  </si>
-  <si>
-    <t>2012-10-06</t>
-  </si>
-  <si>
-    <t>STOPRULE</t>
-  </si>
-  <si>
-    <t>Study Stop Rules</t>
-  </si>
-  <si>
-    <t>NONE</t>
-  </si>
-  <si>
-    <t>C98388</t>
-  </si>
-  <si>
-    <t>TBLIND</t>
-  </si>
-  <si>
-    <t>Trial Blinding Schema</t>
-  </si>
-  <si>
-    <t>DOUBLE BLIND</t>
-  </si>
-  <si>
-    <t>C15228</t>
-  </si>
-  <si>
-    <t>TCNTRL</t>
-  </si>
-  <si>
-    <t>Control Type</t>
-  </si>
-  <si>
-    <t>C49648</t>
-  </si>
-  <si>
-    <t>TDIGRP</t>
-  </si>
-  <si>
-    <t>Diagnosis Group</t>
-  </si>
-  <si>
-    <t>TINDTP</t>
-  </si>
-  <si>
-    <t>Trial Intent Type</t>
-  </si>
-  <si>
-    <t>TREATMENT</t>
-  </si>
-  <si>
-    <t>C49656</t>
-  </si>
-  <si>
-    <t>TITLE</t>
-  </si>
-  <si>
-    <t>Trial Title</t>
-  </si>
-  <si>
-    <t>Safety and Efficacy of Zanomaline in Patients with Mild to Moderate Alzheimers Disease.</t>
-  </si>
-  <si>
-    <t>TPHASE</t>
-  </si>
-  <si>
-    <t>Trial Phase Classification</t>
-  </si>
-  <si>
-    <t>PHASE II TRIAL</t>
-  </si>
-  <si>
-    <t>C15601</t>
-  </si>
-  <si>
     <t>0XXX0X00XX</t>
   </si>
   <si>
@@ -638,10 +641,6 @@
   </si>
   <si>
     <t>C49666</t>
-  </si>
-  <si>
-    <t>TSSEQ</t>
-    <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -683,7 +682,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -700,20 +699,8 @@
         <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -721,26 +708,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9D9D9"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -748,13 +720,6 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1155,10 +1120,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="5" max="5" width="31.5546875" customWidth="1"/>
+    <col min="5" max="5" width="29.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1214,12 +1179,10 @@
       <c r="D3" s="2">
         <v>46</v>
       </c>
-      <c r="E3" s="9" t="s">
-        <v>205</v>
-      </c>
-      <c r="F3" s="2">
-        <v>1</v>
-      </c>
+      <c r="E3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="5"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="2">
@@ -1235,10 +1198,10 @@
         <v>46</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1252,13 +1215,13 @@
         <v>14</v>
       </c>
       <c r="D5" s="2">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
+      </c>
+      <c r="F5" s="2">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1275,9 +1238,11 @@
         <v>53</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" s="5"/>
+        <v>15</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="2">
@@ -1292,18 +1257,34 @@
       <c r="D7" s="2">
         <v>53</v>
       </c>
-      <c r="E7" s="9" t="s">
-        <v>205</v>
-      </c>
-      <c r="F7" s="2">
-        <v>1</v>
-      </c>
+      <c r="E7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="2">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="2">
+        <v>53</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:F2 A4:F4 B5:F5" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:F2 A4:F6 A3:E3 A8:E8 A7:E7" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1312,35 +1293,31 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K55"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
-  <cols>
-    <col min="6" max="6" width="44.5546875" customWidth="1"/>
-    <col min="7" max="7" width="28.33203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="D1" s="1" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>15</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>28</v>
@@ -1468,16 +1445,16 @@
         <v>1</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -1491,28 +1468,28 @@
         <v>1</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H6" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I6" s="2" t="s">
+      <c r="J6" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="K6" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -1526,28 +1503,28 @@
         <v>1</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E7" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="G7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I7" s="2" t="s">
+      <c r="J7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="K7" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1561,19 +1538,19 @@
         <v>1</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1587,25 +1564,25 @@
         <v>1</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -1619,16 +1596,16 @@
         <v>1</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -1642,25 +1619,25 @@
         <v>1</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E11" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>71</v>
-      </c>
       <c r="H11" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -1674,16 +1651,16 @@
         <v>1</v>
       </c>
       <c r="D12" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -1697,16 +1674,16 @@
         <v>2</v>
       </c>
       <c r="D13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -1720,16 +1697,16 @@
         <v>3</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E14" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="G14" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -1740,19 +1717,19 @@
         <v>45</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -1766,28 +1743,28 @@
         <v>1</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E16" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="H16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I16" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="H16" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>84</v>
-      </c>
       <c r="J16" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K16" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -1801,28 +1778,28 @@
         <v>1</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E17" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="H17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I17" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H17" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>88</v>
-      </c>
       <c r="J17" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K17" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -1836,28 +1813,28 @@
         <v>1</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E18" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="G18" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="H18" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I18" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="H18" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>92</v>
-      </c>
       <c r="J18" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K18" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -1871,25 +1848,25 @@
         <v>1</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E19" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="H19" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -1903,28 +1880,28 @@
         <v>1</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E20" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="F20" s="2" t="s">
-        <v>98</v>
-      </c>
       <c r="G20" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I20" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H20" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I20" s="2" t="s">
+      <c r="J20" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="J20" s="2" t="s">
+      <c r="K20" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K20" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -1938,28 +1915,28 @@
         <v>1</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E21" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="G21" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="H21" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I21" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="H21" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I21" s="2" t="s">
+      <c r="J21" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="J21" s="2" t="s">
+      <c r="K21" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -1973,28 +1950,28 @@
         <v>1</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E22" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="G22" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="H22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I22" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="H22" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>108</v>
-      </c>
       <c r="J22" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K22" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K22" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -2008,28 +1985,28 @@
         <v>1</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E23" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="G23" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="G23" s="2" t="s">
+      <c r="H23" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I23" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="H23" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>112</v>
-      </c>
       <c r="J23" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K23" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -2043,25 +2020,25 @@
         <v>1</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E24" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="G24" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="G24" s="2" t="s">
-        <v>115</v>
-      </c>
       <c r="H24" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -2075,16 +2052,16 @@
         <v>1</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E25" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F25" s="2" t="s">
-        <v>117</v>
-      </c>
       <c r="G25" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -2098,16 +2075,16 @@
         <v>1</v>
       </c>
       <c r="D26" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="F26" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="G26" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -2121,16 +2098,16 @@
         <v>2</v>
       </c>
       <c r="D27" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="G27" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -2144,16 +2121,16 @@
         <v>1</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E28" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="G28" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -2167,16 +2144,16 @@
         <v>2</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E29" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="F29" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F29" s="2" t="s">
-        <v>125</v>
-      </c>
       <c r="G29" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -2187,19 +2164,19 @@
         <v>45</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E30" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F30" s="2" t="s">
-        <v>125</v>
-      </c>
       <c r="G30" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -2210,19 +2187,19 @@
         <v>45</v>
       </c>
       <c r="C31" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="G31" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -2233,19 +2210,19 @@
         <v>45</v>
       </c>
       <c r="C32" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="G32" s="2" t="s">
         <v>131</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -2259,25 +2236,25 @@
         <v>1</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E33" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="G33" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="H33" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I33" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="H33" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I33" s="2" t="s">
+      <c r="J33" s="2" t="s">
         <v>136</v>
-      </c>
-      <c r="J33" s="2" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -2291,16 +2268,16 @@
         <v>1</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E34" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="G34" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -2314,28 +2291,28 @@
         <v>1</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E35" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="F35" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="G35" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="H35" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I35" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="H35" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I35" s="2" t="s">
-        <v>144</v>
-      </c>
       <c r="J35" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K35" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K35" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -2349,16 +2326,16 @@
         <v>1</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E36" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="F36" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="F36" s="2" t="s">
+      <c r="G36" s="2" t="s">
         <v>146</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -2372,25 +2349,25 @@
         <v>1</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E37" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="F37" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="F37" s="2" t="s">
+      <c r="G37" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="G37" s="2" t="s">
+      <c r="H37" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="J37" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I37" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="J37" s="2" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -2404,28 +2381,28 @@
         <v>1</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E38" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="F38" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F38" s="2" t="s">
+      <c r="G38" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="G38" s="2" t="s">
+      <c r="H38" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I38" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="H38" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I38" s="2" t="s">
-        <v>155</v>
-      </c>
       <c r="J38" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K38" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K38" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -2439,16 +2416,16 @@
         <v>1</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E39" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="F39" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="F39" s="2" t="s">
+      <c r="G39" s="2" t="s">
         <v>157</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -2462,16 +2439,16 @@
         <v>1</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E40" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="F40" s="2" t="s">
+      <c r="G40" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -2485,25 +2462,25 @@
         <v>1</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E41" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="F41" s="2" t="s">
+      <c r="G41" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="G41" s="2" t="s">
-        <v>164</v>
-      </c>
       <c r="H41" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="42" spans="1:11">
@@ -2517,28 +2494,28 @@
         <v>1</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E42" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="F42" s="2" t="s">
+      <c r="G42" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="G42" s="2" t="s">
+      <c r="H42" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I42" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="H42" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I42" s="2" t="s">
-        <v>168</v>
-      </c>
       <c r="J42" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K42" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K42" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -2552,16 +2529,16 @@
         <v>1</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E43" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="F43" s="2" t="s">
+      <c r="G43" s="2" t="s">
         <v>170</v>
-      </c>
-      <c r="G43" s="2" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -2575,25 +2552,25 @@
         <v>1</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E44" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="F44" s="2" t="s">
+      <c r="G44" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="G44" s="2" t="s">
-        <v>174</v>
-      </c>
       <c r="H44" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -2607,16 +2584,16 @@
         <v>1</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E45" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F45" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="F45" s="2" t="s">
+      <c r="G45" s="2" t="s">
         <v>176</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -2626,32 +2603,32 @@
       <c r="B46" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C46" s="8">
-        <v>1</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="E46" s="7" t="s">
+      <c r="C46" s="2">
+        <v>1</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E46" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F46" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G46" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H46" s="6" t="s">
-        <v>46</v>
+      <c r="F46" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="I46" s="2" t="s">
         <v>178</v>
       </c>
       <c r="J46" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K46" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K46" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -2665,7 +2642,7 @@
         <v>1</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>179</v>
@@ -2677,16 +2654,16 @@
         <v>181</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="I47" s="2" t="s">
         <v>182</v>
       </c>
       <c r="J47" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K47" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K47" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="48" spans="1:11">
@@ -2700,7 +2677,7 @@
         <v>1</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>183</v>
@@ -2709,19 +2686,19 @@
         <v>184</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="I48" s="2" t="s">
         <v>185</v>
       </c>
       <c r="J48" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K48" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K48" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="49" spans="1:11">
@@ -2735,7 +2712,7 @@
         <v>1</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>186</v>
@@ -2755,7 +2732,7 @@
         <v>1</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>188</v>
@@ -2767,16 +2744,16 @@
         <v>190</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="I50" s="2" t="s">
         <v>191</v>
       </c>
       <c r="J50" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K50" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K50" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="51" spans="1:11">
@@ -2790,7 +2767,7 @@
         <v>1</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>192</v>
@@ -2813,7 +2790,7 @@
         <v>1</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>195</v>
@@ -2825,16 +2802,16 @@
         <v>197</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="I52" s="2" t="s">
         <v>198</v>
       </c>
       <c r="J52" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K52" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K52" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="53" spans="1:11">
@@ -2844,27 +2821,29 @@
       <c r="B53" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C53" s="8">
-        <v>1</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>46</v>
+      <c r="C53" s="2">
+        <v>1</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>22</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F53" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="G53" s="10"/>
-      <c r="H53" s="6" t="s">
-        <v>46</v>
+        <v>21</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G53" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="54" spans="1:11">
@@ -2878,28 +2857,28 @@
         <v>1</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="J54" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K54" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K54" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="55" spans="1:11">
@@ -2910,38 +2889,38 @@
         <v>45</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="J55" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K55" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="K55" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:K52 A54:K55 A53:F53 H53:K53" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:K55" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>